<commit_message>
He completado 10 casos de prueba de registros
</commit_message>
<xml_diff>
--- a/casos_de_prueba/matriz_pruebas.xlsx
+++ b/casos_de_prueba/matriz_pruebas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\OneDrive\Escritorio\QA\ProyectoFinal-BelenFn\casos_de_prueba\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7DCF31F-9AE0-4DF2-B99D-BD507894387A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32EB1B06-C827-4132-B211-FA120A5C3E66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="79">
   <si>
     <t>Nombre del Proyecto:</t>
   </si>
@@ -69,19 +69,7 @@
     <t>Flujo correcto</t>
   </si>
   <si>
-    <t>Usuario logueado</t>
-  </si>
-  <si>
-    <t>Módulos conectados</t>
-  </si>
-  <si>
-    <t>1. Login 2. Navegar</t>
-  </si>
-  <si>
     <t>Media</t>
-  </si>
-  <si>
-    <t>Sesión válida</t>
   </si>
   <si>
     <t>Descripción</t>
@@ -167,22 +155,154 @@
     <t>Registro con email inválido</t>
   </si>
   <si>
-    <t>1.Ingresar email sin formato correcto
-2.Ingresar contraseña válida</t>
-  </si>
-  <si>
-    <t>Mostrar mensaje de error 
-de email inválido</t>
-  </si>
-  <si>
     <t>Registro con contraseña 
 menor a 8 caracteres</t>
   </si>
   <si>
-    <t>Mostrar mensaje de validación</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
+    <t>Registro con campos vacíos</t>
+  </si>
+  <si>
+    <t>Registro con email ya
+existente</t>
+  </si>
+  <si>
+    <t>Registro con espacios 
+en blanco en email</t>
+  </si>
+  <si>
+    <t>Registro con contraseña 
+válida pero sin 
+confirmación correcta</t>
+  </si>
+  <si>
+    <t>Registro con caracteres 
+especiales en contraseña</t>
+  </si>
+  <si>
+    <t>Registro cancelado
+ antes de enviar</t>
+  </si>
+  <si>
+    <t>Validación de mensaje 
+de confirmación exitoso</t>
+  </si>
+  <si>
+    <t>Mostrar mensaje de error
+"Email inválido"</t>
+  </si>
+  <si>
+    <t>Validación de formato</t>
+  </si>
+  <si>
+    <t>CP-01</t>
+  </si>
+  <si>
+    <t>1.Ingresar email sin formato correcto (ejemplo: belen.com)
+2.Ingresar contraseña válida
+3.Presionar "Registrarse"</t>
+  </si>
+  <si>
+    <t>1.Ingresar email valido
+2.Ingresar contraseña de menos de 8 caracteres
+3.Presionar "Registrarse"</t>
+  </si>
+  <si>
+    <t>Mostrar mensaje de 
+validación de contraseña</t>
+  </si>
+  <si>
+    <t>Regla de seguridad mínima</t>
+  </si>
+  <si>
+    <t>1.Dejar campos vacíos 
+2.Presionar "Registrarse"</t>
+  </si>
+  <si>
+    <t>No permitir registro y 
+mostrar mensaje de campos obligatorios</t>
+  </si>
+  <si>
+    <t>Validación obligatoria</t>
+  </si>
+  <si>
+    <t>Email ya registrado 
+en el sistema</t>
+  </si>
+  <si>
+    <t>1. Ingresar email ya existente
+2.Ingresar contraseña válida
+3.Presionar "Registrarse"</t>
+  </si>
+  <si>
+    <t>Mostrar mensaje
+"Usuario ya existente"</t>
+  </si>
+  <si>
+    <t>Validación de duplicados</t>
+  </si>
+  <si>
+    <t>1.Ingresar " usuario@email.com
+ " (con espacios)
+2.Ingresar contraseña válida
+3.Presionar "Registrarse"</t>
+  </si>
+  <si>
+    <t>El sistema elimina espacios 
+o muestra error de validación</t>
+  </si>
+  <si>
+    <t>1. Ingresar email válido
+2. Ingresar contraseña válida
+3. Ingresar confirmación diferente
+4. Presionar "Registrarse"</t>
+  </si>
+  <si>
+    <t>Mostrar mensaje
+"Las contraseñas no coinciden"</t>
+  </si>
+  <si>
+    <t>Validación de coincidencia</t>
+  </si>
+  <si>
+    <t>1. Ingresar email válido
+2. Ingresar contraseña con caracteres especiales (Ej: Pass@1234)
+3. Confirmar contraseña
+4.Presionar "Registrarse"</t>
+  </si>
+  <si>
+    <t>Permitir registro exitoso</t>
+  </si>
+  <si>
+    <t>Baja</t>
+  </si>
+  <si>
+    <t>Validación de seguridad</t>
+  </si>
+  <si>
+    <t>1. Ingresar datos
+2. Presionar botón "Cancelar"</t>
+  </si>
+  <si>
+    <t>Usuario en pantalla 
+de registro</t>
+  </si>
+  <si>
+    <t>Regresar a pantalla 
+anterior sin guardar datos</t>
+  </si>
+  <si>
+    <t>Flujo alternativo</t>
+  </si>
+  <si>
+    <t>1. Completar registro válido
+2. Observar mensaje mostrado</t>
+  </si>
+  <si>
+    <t>Mostrar mensaje 
+"Registro exitoso" visible y claro</t>
+  </si>
+  <si>
+    <t>Validación visual</t>
   </si>
 </sst>
 </file>
@@ -212,7 +332,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -331,27 +451,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -361,44 +467,53 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="14">
+  <dxfs count="15">
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
-        <left/>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
         <right style="thin">
           <color indexed="64"/>
         </right>
@@ -408,11 +523,19 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
       </border>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
@@ -425,7 +548,8 @@
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -436,12 +560,11 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -454,12 +577,11 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -472,12 +594,11 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -490,12 +611,11 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -508,12 +628,11 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -526,12 +645,11 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -544,15 +662,12 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
         <right style="thin">
           <color indexed="64"/>
         </right>
@@ -562,12 +677,11 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right style="thin">
           <color indexed="64"/>
@@ -578,8 +692,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -591,6 +703,15 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
@@ -598,15 +719,6 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
@@ -626,19 +738,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A134B595-C49F-4EAC-8FFC-B42C7BB2A632}" name="Tabla2" displayName="Tabla2" ref="A5:J15" totalsRowShown="0" headerRowDxfId="1" headerRowBorderDxfId="12" tableBorderDxfId="13" totalsRowBorderDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A134B595-C49F-4EAC-8FFC-B42C7BB2A632}" name="Tabla2" displayName="Tabla2" ref="A5:J15" totalsRowShown="0" headerRowDxfId="2" dataDxfId="1" headerRowBorderDxfId="14" tableBorderDxfId="13" totalsRowBorderDxfId="12">
   <autoFilter ref="A5:J15" xr:uid="{A134B595-C49F-4EAC-8FFC-B42C7BB2A632}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{9D81CB4B-CA0A-4EE0-A03F-853D8109B5F1}" name="ID" dataDxfId="10"/>
-    <tableColumn id="10" xr3:uid="{D2C658D0-832C-49E8-95A9-74ADCB4387B3}" name="Historia" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{C7D855B1-B74B-4F87-B517-4FA3028A2CE7}" name="Descripción" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{5B761194-0897-4090-BC1C-735E6430ABC1}" name="Precondiciones" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{3C066711-FAAE-4423-83AD-90F312BD19E6}" name="Pasos" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{664E6974-C33B-4B99-81A3-32B7D066FD96}" name="Resultado esperado" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{7AEF72FF-6D41-48F0-9F15-2F0B1931A4CA}" name="Resultado obtenido" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{3165D225-7B86-4C0F-86CB-84D9DB89811B}" name="Prioridad" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{68F9A74B-4D4E-4101-B03C-4044C85E3436}" name="Severidad" dataDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{127484FB-2EE3-42FE-8DF9-00035A357AF2}" name="Observaciones" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{9D81CB4B-CA0A-4EE0-A03F-853D8109B5F1}" name="ID" dataDxfId="11"/>
+    <tableColumn id="10" xr3:uid="{D2C658D0-832C-49E8-95A9-74ADCB4387B3}" name="Historia" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{C7D855B1-B74B-4F87-B517-4FA3028A2CE7}" name="Descripción" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{5B761194-0897-4090-BC1C-735E6430ABC1}" name="Precondiciones" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{3C066711-FAAE-4423-83AD-90F312BD19E6}" name="Pasos" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{664E6974-C33B-4B99-81A3-32B7D066FD96}" name="Resultado esperado" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{7AEF72FF-6D41-48F0-9F15-2F0B1931A4CA}" name="Resultado obtenido" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{3165D225-7B86-4C0F-86CB-84D9DB89811B}" name="Prioridad" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{68F9A74B-4D4E-4101-B03C-4044C85E3436}" name="Severidad" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{127484FB-2EE3-42FE-8DF9-00035A357AF2}" name="Observaciones" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -911,14 +1023,14 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="11.6328125" customWidth="1"/>
-    <col min="3" max="3" width="22.90625" customWidth="1"/>
+    <col min="3" max="3" width="25.26953125" customWidth="1"/>
     <col min="4" max="4" width="21.1796875" customWidth="1"/>
     <col min="5" max="5" width="23.453125" customWidth="1"/>
     <col min="6" max="6" width="31" customWidth="1"/>
-    <col min="7" max="7" width="10.54296875" customWidth="1"/>
+    <col min="7" max="7" width="20.90625" customWidth="1"/>
     <col min="8" max="8" width="11" customWidth="1"/>
     <col min="9" max="9" width="22.81640625" customWidth="1"/>
-    <col min="10" max="10" width="17.08984375" customWidth="1"/>
+    <col min="10" max="10" width="23.36328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
@@ -937,241 +1049,357 @@
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="5"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="4"/>
       <c r="E2" s="1" t="s">
         <v>3</v>
       </c>
       <c r="F2" s="1"/>
     </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+    </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="9" t="s">
+      <c r="B5" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="H5" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="I5" s="9" t="s">
+      <c r="H5" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="I5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="J5" s="10" t="s">
+      <c r="J5" s="8" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="I6" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="J6" s="9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="87" x14ac:dyDescent="0.35">
+      <c r="A7" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="F7" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="G7" s="9"/>
+      <c r="H7" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="I7" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+      <c r="A8" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="I8" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="F9" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="I9" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A10" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E6" s="13" t="s">
+      <c r="B10" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="F6" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2" t="s">
+      <c r="D10" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="F10" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="J6" s="2" t="s">
-        <v>12</v>
+      <c r="I10" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>62</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A7" s="14" t="s">
+    <row r="11" spans="1:10" ht="87" x14ac:dyDescent="0.35">
+      <c r="A11" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B11" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C11" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D11" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="F11" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="I11" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="87" x14ac:dyDescent="0.35">
+      <c r="A12" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="D12" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="F12" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="I12" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="J12" s="5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="87" x14ac:dyDescent="0.35">
+      <c r="A13" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J7" s="15" t="s">
-        <v>14</v>
+      <c r="D13" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I13" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="J13" s="5" t="s">
+        <v>71</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A8" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="C8" s="17" t="s">
+    <row r="14" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A14" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="D14" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="F14" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="I14" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="J14" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+      <c r="A15" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="F15" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="F8" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="G8" s="18"/>
-      <c r="H8" s="18"/>
-      <c r="I8" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="J8" s="19" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A9" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="7"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A10" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B10" t="s">
-        <v>34</v>
-      </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="J10" s="7"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A11" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-      <c r="J11" s="7"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A12" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
-      <c r="J12" s="7"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A13" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="7"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A14" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B14" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-      <c r="J14" s="7"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A15" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-      <c r="J15" s="7"/>
+      <c r="I15" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="J15" s="5" t="s">
+        <v>78</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Actualizo matriz de pruebas y reporte de bugs
</commit_message>
<xml_diff>
--- a/casos_de_prueba/matriz_pruebas.xlsx
+++ b/casos_de_prueba/matriz_pruebas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\OneDrive\Escritorio\QA\ProyectoFinal-BelenFn\casos_de_prueba\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{019DBF40-3E17-45CF-9BF8-C98FD7227106}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CB40249-D748-4482-AC7C-33E520A05838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -818,15 +818,6 @@
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -845,11 +836,39 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="16">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
@@ -1059,22 +1078,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right style="thin">
@@ -1112,10 +1115,26 @@
       </border>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <border outline="0">
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
   </dxfs>
@@ -1132,19 +1151,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A134B595-C49F-4EAC-8FFC-B42C7BB2A632}" name="Tabla2" displayName="Tabla2" ref="A5:J35" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9" headerRowBorderDxfId="14" tableBorderDxfId="13" totalsRowBorderDxfId="12">
-  <autoFilter ref="A5:J35" xr:uid="{A134B595-C49F-4EAC-8FFC-B42C7BB2A632}"/>
-  <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{9D81CB4B-CA0A-4EE0-A03F-853D8109B5F1}" name="ID" dataDxfId="11"/>
-    <tableColumn id="10" xr3:uid="{D2C658D0-832C-49E8-95A9-74ADCB4387B3}" name="Historia" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{C7D855B1-B74B-4F87-B517-4FA3028A2CE7}" name="Descripción" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{5B761194-0897-4090-BC1C-735E6430ABC1}" name="Precondiciones" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{3C066711-FAAE-4423-83AD-90F312BD19E6}" name="Pasos" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{664E6974-C33B-4B99-81A3-32B7D066FD96}" name="Resultado esperado" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{7AEF72FF-6D41-48F0-9F15-2F0B1931A4CA}" name="Resultado obtenido" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{3165D225-7B86-4C0F-86CB-84D9DB89811B}" name="Prioridad" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{68F9A74B-4D4E-4101-B03C-4044C85E3436}" name="Severidad" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{127484FB-2EE3-42FE-8DF9-00035A357AF2}" name="Observaciones" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A134B595-C49F-4EAC-8FFC-B42C7BB2A632}" name="Tabla2" displayName="Tabla2" ref="A5:K35" totalsRowShown="0" headerRowDxfId="15" dataDxfId="13" headerRowBorderDxfId="14" tableBorderDxfId="12" totalsRowBorderDxfId="11">
+  <autoFilter ref="A5:K35" xr:uid="{A134B595-C49F-4EAC-8FFC-B42C7BB2A632}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{9D81CB4B-CA0A-4EE0-A03F-853D8109B5F1}" name="ID" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{D2C658D0-832C-49E8-95A9-74ADCB4387B3}" name="Historia" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{C7D855B1-B74B-4F87-B517-4FA3028A2CE7}" name="Descripción" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{5B761194-0897-4090-BC1C-735E6430ABC1}" name="Precondiciones" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{3C066711-FAAE-4423-83AD-90F312BD19E6}" name="Pasos" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{664E6974-C33B-4B99-81A3-32B7D066FD96}" name="Resultado esperado" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{7AEF72FF-6D41-48F0-9F15-2F0B1931A4CA}" name="Resultado obtenido" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{3165D225-7B86-4C0F-86CB-84D9DB89811B}" name="Prioridad" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{68F9A74B-4D4E-4101-B03C-4044C85E3436}" name="Severidad" dataDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{127484FB-2EE3-42FE-8DF9-00035A357AF2}" name="Observaciones" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{4EE2CC9E-54AB-48CF-B7F5-6D35CDB3E83A}" name="Estado" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1425,7 +1445,7 @@
     <col min="8" max="8" width="11" customWidth="1"/>
     <col min="9" max="9" width="22.81640625" customWidth="1"/>
     <col min="10" max="10" width="23.36328125" customWidth="1"/>
-    <col min="11" max="11" width="22.81640625" customWidth="1"/>
+    <col min="11" max="11" width="16.26953125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.35">
@@ -1444,931 +1464,930 @@
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="4"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="10"/>
       <c r="E2" s="1" t="s">
         <v>3</v>
       </c>
       <c r="F2" s="1"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="J5" s="7" t="s">
+      <c r="J5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="K5" s="7" t="s">
+      <c r="K5" s="4" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="G6" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="I6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="J6" s="8" t="s">
+      <c r="J6" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="K6" s="4" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="I7" s="7" t="s">
+      <c r="I7" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="J7" s="8" t="s">
+      <c r="J7" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="K7" s="7" t="s">
+      <c r="K7" s="4" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="I8" s="7" t="s">
+      <c r="I8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="J8" s="8" t="s">
+      <c r="J8" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="K8" s="7" t="s">
+      <c r="K8" s="4" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="H9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="I9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="J9" s="8" t="s">
+      <c r="J9" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="K9" s="7" t="s">
+      <c r="K9" s="4" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="I10" s="7" t="s">
+      <c r="I10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="J10" s="8" t="s">
+      <c r="J10" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="K10" s="7" t="s">
+      <c r="K10" s="4" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="G11" s="8" t="s">
+      <c r="G11" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="H11" s="7" t="s">
+      <c r="H11" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="7" t="s">
+      <c r="I11" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="J11" s="8" t="s">
+      <c r="J11" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="K11" s="7" t="s">
+      <c r="K11" s="4" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="87" x14ac:dyDescent="0.35">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G12" s="8" t="s">
+      <c r="G12" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="I12" s="7" t="s">
+      <c r="I12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="J12" s="8" t="s">
+      <c r="J12" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="K12" s="7" t="s">
+      <c r="K12" s="4" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="87" x14ac:dyDescent="0.35">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="G13" s="8" t="s">
+      <c r="G13" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="H13" s="7" t="s">
+      <c r="H13" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="I13" s="7" t="s">
+      <c r="I13" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="J13" s="8" t="s">
+      <c r="J13" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="K13" s="7" t="s">
+      <c r="K13" s="4" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="G14" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="H14" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="I14" s="7" t="s">
+      <c r="I14" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="J14" s="8" t="s">
+      <c r="J14" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="K14" s="7" t="s">
+      <c r="K14" s="4" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="G15" s="8" t="s">
+      <c r="G15" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="H15" s="7" t="s">
+      <c r="H15" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="7" t="s">
+      <c r="I15" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="J15" s="8" t="s">
+      <c r="J15" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="K15" s="7" t="s">
+      <c r="K15" s="4" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="87" x14ac:dyDescent="0.35">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="E16" s="8" t="s">
+      <c r="E16" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="G16" s="7" t="s">
+      <c r="G16" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="H16" s="7" t="s">
+      <c r="H16" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="I16" s="7" t="s">
+      <c r="I16" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="J16" s="8" t="s">
+      <c r="J16" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="K16" s="7" t="s">
+      <c r="K16" s="4" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="G17" s="8" t="s">
+      <c r="G17" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="H17" s="7" t="s">
+      <c r="H17" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="I17" s="7" t="s">
+      <c r="I17" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="J17" s="8" t="s">
+      <c r="J17" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="K17" s="7" t="s">
+      <c r="K17" s="4" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="87" x14ac:dyDescent="0.35">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="E18" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="F18" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="G18" s="8" t="s">
+      <c r="G18" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="H18" s="7" t="s">
+      <c r="H18" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="I18" s="7" t="s">
+      <c r="I18" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="J18" s="8" t="s">
+      <c r="J18" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="K18" s="7" t="s">
+      <c r="K18" s="4" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D19" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="E19" s="8" t="s">
+      <c r="E19" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="F19" s="8" t="s">
+      <c r="F19" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="G19" s="8" t="s">
+      <c r="G19" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="H19" s="7" t="s">
+      <c r="H19" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="I19" s="7" t="s">
+      <c r="I19" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="J19" s="8" t="s">
+      <c r="J19" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="K19" s="7" t="s">
+      <c r="K19" s="4" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="E20" s="8" t="s">
+      <c r="E20" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="F20" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="G20" s="8" t="s">
+      <c r="G20" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="H20" s="7" t="s">
+      <c r="H20" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="I20" s="7" t="s">
+      <c r="I20" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="J20" s="8" t="s">
+      <c r="J20" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="K20" s="7" t="s">
+      <c r="K20" s="4" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="87" x14ac:dyDescent="0.35">
+      <c r="A21" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="J21" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="116" x14ac:dyDescent="0.35">
+      <c r="A22" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G22" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="J22" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A23" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="J23" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="K23" s="4" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="87" x14ac:dyDescent="0.35">
-      <c r="A21" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="D21" s="7" t="s">
+    <row r="24" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A24" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D24" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="E21" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="F21" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="G21" s="8" t="s">
-        <v>176</v>
-      </c>
-      <c r="H21" s="7" t="s">
+      <c r="E24" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="I24" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="J24" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="K24" s="4" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+      <c r="A25" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="G25" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="H25" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="I21" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="J21" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="K21" s="7" t="s">
+      <c r="I25" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="J25" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="K25" s="4" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="116" x14ac:dyDescent="0.35">
-      <c r="A22" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="E22" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="F22" s="8" t="s">
-        <v>156</v>
-      </c>
-      <c r="G22" s="8" t="s">
-        <v>177</v>
-      </c>
-      <c r="H22" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="I22" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="J22" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="K22" s="7" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A23" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="E23" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="F23" s="8" t="s">
-        <v>158</v>
-      </c>
-      <c r="G23" s="8" t="s">
-        <v>178</v>
-      </c>
-      <c r="H23" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="I23" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="J23" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="K23" s="7" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A24" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="C24" s="8" t="s">
-        <v>160</v>
-      </c>
-      <c r="D24" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="E24" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="F24" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="G24" s="8" t="s">
-        <v>179</v>
-      </c>
-      <c r="H24" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="I24" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="J24" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="K24" s="7" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="A25" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>146</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="F25" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="G25" s="8" t="s">
-        <v>180</v>
-      </c>
-      <c r="H25" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="I25" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="J25" s="8" t="s">
-        <v>171</v>
-      </c>
-      <c r="K25" s="7" t="s">
-        <v>183</v>
-      </c>
-    </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A26" s="9" t="s">
+      <c r="A26" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
-      <c r="F26" s="7"/>
-      <c r="G26" s="7"/>
-      <c r="H26" s="7"/>
-      <c r="I26" s="7"/>
-      <c r="J26" s="7"/>
-      <c r="K26" s="7"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="4"/>
+      <c r="J26" s="4"/>
+      <c r="K26" s="4"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A27" s="9" t="s">
+      <c r="A27" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C27" s="7"/>
-      <c r="D27" s="7"/>
-      <c r="E27" s="7"/>
-      <c r="F27" s="7"/>
-      <c r="G27" s="7"/>
-      <c r="H27" s="7"/>
-      <c r="I27" s="7"/>
-      <c r="J27" s="7"/>
-      <c r="K27" s="7"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
+      <c r="H27" s="4"/>
+      <c r="I27" s="4"/>
+      <c r="J27" s="4"/>
+      <c r="K27" s="4"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A28" s="9" t="s">
+      <c r="A28" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7"/>
-      <c r="E28" s="7"/>
-      <c r="F28" s="7"/>
-      <c r="G28" s="7"/>
-      <c r="H28" s="7"/>
-      <c r="I28" s="7"/>
-      <c r="J28" s="7"/>
-      <c r="K28" s="7"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+      <c r="G28" s="4"/>
+      <c r="H28" s="4"/>
+      <c r="I28" s="4"/>
+      <c r="J28" s="4"/>
+      <c r="K28" s="4"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A29" s="9" t="s">
+      <c r="A29" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="B29" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="C29" s="7"/>
-      <c r="D29" s="7"/>
-      <c r="E29" s="7"/>
-      <c r="F29" s="7"/>
-      <c r="G29" s="7"/>
-      <c r="H29" s="7"/>
-      <c r="I29" s="7"/>
-      <c r="J29" s="7"/>
-      <c r="K29" s="7"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="4"/>
+      <c r="K29" s="4"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A30" s="9" t="s">
+      <c r="A30" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="C30" s="7"/>
-      <c r="D30" s="7"/>
-      <c r="E30" s="7"/>
-      <c r="F30" s="7"/>
-      <c r="G30" s="7"/>
-      <c r="H30" s="7"/>
-      <c r="I30" s="7"/>
-      <c r="J30" s="7"/>
-      <c r="K30" s="7"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
+      <c r="F30" s="4"/>
+      <c r="G30" s="4"/>
+      <c r="H30" s="4"/>
+      <c r="I30" s="4"/>
+      <c r="J30" s="4"/>
+      <c r="K30" s="4"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A31" s="9" t="s">
+      <c r="A31" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="B31" s="7" t="s">
+      <c r="B31" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="C31" s="7"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
-      <c r="F31" s="7"/>
-      <c r="G31" s="7"/>
-      <c r="H31" s="7"/>
-      <c r="I31" s="7"/>
-      <c r="J31" s="7"/>
-      <c r="K31" s="7"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
+      <c r="H31" s="4"/>
+      <c r="I31" s="4"/>
+      <c r="J31" s="4"/>
+      <c r="K31" s="4"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A32" s="9" t="s">
+      <c r="A32" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="B32" s="7" t="s">
+      <c r="B32" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="C32" s="7"/>
-      <c r="D32" s="7"/>
-      <c r="E32" s="7"/>
-      <c r="F32" s="7"/>
-      <c r="G32" s="7"/>
-      <c r="H32" s="7"/>
-      <c r="I32" s="7"/>
-      <c r="J32" s="7"/>
-      <c r="K32" s="7"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+      <c r="F32" s="4"/>
+      <c r="G32" s="4"/>
+      <c r="H32" s="4"/>
+      <c r="I32" s="4"/>
+      <c r="J32" s="4"/>
+      <c r="K32" s="4"/>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A33" s="9" t="s">
+      <c r="A33" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="B33" s="7" t="s">
+      <c r="B33" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="C33" s="7"/>
-      <c r="D33" s="7"/>
-      <c r="E33" s="7"/>
-      <c r="F33" s="7"/>
-      <c r="G33" s="7"/>
-      <c r="H33" s="7"/>
-      <c r="I33" s="7"/>
-      <c r="J33" s="7"/>
-      <c r="K33" s="7"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="4"/>
+      <c r="H33" s="4"/>
+      <c r="I33" s="4"/>
+      <c r="J33" s="4"/>
+      <c r="K33" s="4"/>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A34" s="9" t="s">
+      <c r="A34" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="B34" s="7" t="s">
+      <c r="B34" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="C34" s="7"/>
-      <c r="D34" s="7"/>
-      <c r="E34" s="7"/>
-      <c r="F34" s="7"/>
-      <c r="G34" s="7"/>
-      <c r="H34" s="7"/>
-      <c r="I34" s="7"/>
-      <c r="J34" s="7"/>
-      <c r="K34" s="7"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="4"/>
+      <c r="G34" s="4"/>
+      <c r="H34" s="4"/>
+      <c r="I34" s="4"/>
+      <c r="J34" s="4"/>
+      <c r="K34" s="4"/>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A35" s="9" t="s">
+      <c r="A35" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="B35" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="C35" s="7"/>
-      <c r="D35" s="7"/>
-      <c r="E35" s="7"/>
-      <c r="F35" s="7"/>
-      <c r="G35" s="7"/>
-      <c r="H35" s="7"/>
-      <c r="I35" s="7"/>
-      <c r="J35" s="7"/>
-      <c r="K35" s="7"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4"/>
+      <c r="G35" s="4"/>
+      <c r="H35" s="4"/>
+      <c r="I35" s="4"/>
+      <c r="J35" s="4"/>
+      <c r="K35" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2376,7 +2395,7 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="A6:K25">
-    <cfRule type="dataBar" priority="1">
+    <cfRule type="dataBar" priority="3">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>

</xml_diff>